<commit_message>
Refactor: Update join meeting checklist
Co-authored-by: vanttnguyen <vanttnguyen@kms-technology.com>
</commit_message>
<xml_diff>
--- a/Meeting_Collaborative_Beta_JoinMeeting_TestChecklist.xlsx
+++ b/Meeting_Collaborative_Beta_JoinMeeting_TestChecklist.xlsx
@@ -67,103 +67,103 @@
     <t>Host</t>
   </si>
   <si>
-    <t>Host có thể Start/Join session sớm đến 4 giờ trước giờ bắt đầu</t>
-  </si>
-  <si>
-    <t>Session type = Meeting (Collaborative) BETA; Host đã được assign trong Session Editor; Current time = T-4h.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Vào Agenda lobby page
-2) Chọn session
-3) Nhấn Start/Join</t>
-  </si>
-  <si>
-    <t>Host vào được phòng meeting; hiển thị đúng session name/timer; không bị chặn bởi open time attendee.</t>
+    <t>Host can start/join the session up to 4 hours before the scheduled start time</t>
+  </si>
+  <si>
+    <t>Session type = Meeting (Collaborative) BETA; Host is assigned in Session Editor; Current time = T-4h.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Go to Agenda lobby page
+2) Open the session
+3) Click Start/Join</t>
+  </si>
+  <si>
+    <t>Host enters the meeting successfully; correct session title/timer is shown; not blocked by attendee open-time rules.</t>
+  </si>
+  <si>
+    <t>P0</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Not Run</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>JOIN-002</t>
+  </si>
+  <si>
+    <t>Host is blocked when attempting to start/join earlier than 4 hours before start time</t>
+  </si>
+  <si>
+    <t>Session type = Meeting (Collaborative) BETA; Host assigned; Current time = T-4h-1m.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Go to Agenda lobby page
+2) Click Start/Join</t>
+  </si>
+  <si>
+    <t>Host cannot enter; a clear message is shown (e.g., “You can start this session 4 hours before start time”).</t>
+  </si>
+  <si>
+    <t>JOIN-003</t>
+  </si>
+  <si>
+    <t>Attendee</t>
+  </si>
+  <si>
+    <t>Attendee cannot join before the configured attendee open time</t>
+  </si>
+  <si>
+    <t>Attendee open time is configured (e.g., 10 minutes before start); Current time is earlier than open time; Attendee is eligible for the event.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Go to Agenda lobby page
+2) Click Join</t>
+  </si>
+  <si>
+    <t>Attendee is blocked; a message/countdown indicates when the session opens.</t>
+  </si>
+  <si>
+    <t>JOIN-004</t>
+  </si>
+  <si>
+    <t>Attendee can join starting from the configured attendee open time</t>
+  </si>
+  <si>
+    <t>Current time is within the attendee open window; Session is unlocked OR (if locked) a host is available to admit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Go to Agenda lobby page
+2) Click Join
+3) Complete pre-join (if shown)</t>
+  </si>
+  <si>
+    <t>Attendee enters the meeting (or waiting room if locked); no permission/timing gating errors occur.</t>
+  </si>
+  <si>
+    <t>JOIN-005</t>
+  </si>
+  <si>
+    <t>Speaker</t>
+  </si>
+  <si>
+    <t>Speaker join timing follows the intended rule (speaker behaves like attendee or host)</t>
+  </si>
+  <si>
+    <t>Speaker assigned in Session Editor; Attendee open time configured; clarify expected behavior for the product (speaker uses attendee open time vs host early-start).</t>
+  </si>
+  <si>
+    <t>Behavior matches the intended design: speaker is allowed/blocked based on the rule.</t>
   </si>
   <si>
     <t>P1</t>
   </si>
   <si>
-    <t>Functional</t>
-  </si>
-  <si>
-    <t>Not Run</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>JOIN-002</t>
-  </si>
-  <si>
-    <t>Host bị chặn khi cố Start/Join sớm hơn 4 giờ trước giờ bắt đầu</t>
-  </si>
-  <si>
-    <t>Session type = Meeting (Collaborative) BETA; Host assigned; Current time = T-4h-1m.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Vào Agenda lobby page
-2) Nhấn Start/Join</t>
-  </si>
-  <si>
-    <t>Không cho vào phòng; hiển thị thông báo phù hợp (ví dụ: “You can start this session 4 hours before start time”).</t>
-  </si>
-  <si>
-    <t>P0</t>
-  </si>
-  <si>
-    <t>JOIN-003</t>
-  </si>
-  <si>
-    <t>Attendee</t>
-  </si>
-  <si>
-    <t>Attendee không join được trước open time được cấu hình trong Session Editor</t>
-  </si>
-  <si>
-    <t>Open time attendee = (ví dụ) 10 phút trước start; Current time = sớm hơn open time; Attendee đã đăng ký/được phép vào event.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Vào Agenda lobby page
-2) Nhấn Join</t>
-  </si>
-  <si>
-    <t>Attendee bị chặn; hiển thị countdown/label “Opens at …” hoặc message tương đương.</t>
-  </si>
-  <si>
-    <t>JOIN-004</t>
-  </si>
-  <si>
-    <t>Attendee join được đúng từ thời điểm open time trở đi</t>
-  </si>
-  <si>
-    <t>Open time attendee đã đến; Session not locked hoặc nếu locked thì có host để admit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Vào Agenda lobby page
-2) Nhấn Join
-3) Hoàn tất pre-join nếu có</t>
-  </si>
-  <si>
-    <t>Attendee vào được meeting (hoặc vào waiting room nếu locked); không lỗi quyền/time gating.</t>
-  </si>
-  <si>
-    <t>JOIN-005</t>
-  </si>
-  <si>
-    <t>Speaker</t>
-  </si>
-  <si>
-    <t>Speaker join theo rule open time (hoặc rule riêng nếu hệ thống có)</t>
-  </si>
-  <si>
-    <t>Speaker assigned trong Session Editor; Open time configured; xác định behavior kỳ vọng theo product: (a) speaker như attendee hoặc (b) speaker như host.</t>
-  </si>
-  <si>
-    <t>Behavior khớp rule thiết kế: speaker được/không được join sớm tương ứng.</t>
-  </si>
-  <si>
-    <t>Nếu spec chưa rõ, capture behavior thực tế &amp; align với team product.</t>
+    <t>If spec is unclear, capture actual behavior and confirm with product.</t>
   </si>
   <si>
     <t>JOIN-006</t>
@@ -172,18 +172,18 @@
     <t>Agenda Lobby Entry</t>
   </si>
   <si>
-    <t>Join từ Agenda lobby page dẫn đúng vào session phòng meeting</t>
-  </si>
-  <si>
-    <t>Session visible trong Agenda; attendee eligible; open time đã đến.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Mở Agenda
-2) Chọn đúng session
-3) Join</t>
-  </si>
-  <si>
-    <t>Vào đúng session (không nhầm session khác); hiển thị đúng title/time; participant count cập nhật.</t>
+    <t>Joining from the Agenda lobby page routes to the correct meeting session</t>
+  </si>
+  <si>
+    <t>Session is visible on Agenda; attendee is eligible; attendee open time has started.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Open Agenda
+2) Select the correct session
+3) Click Join</t>
+  </si>
+  <si>
+    <t>User lands in the correct session (not another one); correct title/time shown; participant count updates.</t>
   </si>
   <si>
     <t>JOIN-007</t>
@@ -192,17 +192,17 @@
     <t>Unknown/Guest</t>
   </si>
   <si>
-    <t>User chưa đăng nhập/không có quyền bị chặn khi Join</t>
-  </si>
-  <si>
-    <t>User not authenticated hoặc không thuộc event; session visible public link (nếu có).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Truy cập Agenda/Join URL
-2) Thử Join</t>
-  </si>
-  <si>
-    <t>Bị yêu cầu login hoặc hiển thị access denied; không vào được meeting.</t>
+    <t>Unauthenticated or unauthorized user is blocked from joining</t>
+  </si>
+  <si>
+    <t>User is not authenticated OR not part of the event; user has access to a session link (if applicable).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Open Agenda or join URL
+2) Attempt to Join</t>
+  </si>
+  <si>
+    <t>User is prompted to sign in or shown access denied; user cannot enter the meeting.</t>
   </si>
   <si>
     <t>Security</t>
@@ -214,50 +214,50 @@
     <t>Pre-join &amp; Device Checks</t>
   </si>
   <si>
-    <t>Join khi trình duyệt chưa cấp quyền microphone</t>
-  </si>
-  <si>
-    <t>Browser permission mic = blocked; open time đã đến.</t>
+    <t>Join with microphone permission blocked</t>
+  </si>
+  <si>
+    <t>Browser mic permission = blocked; attendee open time has started.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Join meeting
-2) Bật mic trong pre-join hoặc trong meeting</t>
-  </si>
-  <si>
-    <t>App hiển thị prompt/guide cấp quyền; trạng thái mute hiển thị đúng; không crash.</t>
+2) Try to enable microphone in pre-join or in-meeting</t>
+  </si>
+  <si>
+    <t>App shows clear guidance to enable permissions; mute state is correct; meeting does not crash.</t>
   </si>
   <si>
     <t>JOIN-009</t>
   </si>
   <si>
-    <t>Join khi trình duyệt chưa cấp quyền camera</t>
-  </si>
-  <si>
-    <t>Browser permission camera = blocked; open time đã đến.</t>
+    <t>Join with camera permission blocked</t>
+  </si>
+  <si>
+    <t>Browser camera permission = blocked; attendee open time has started.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Join meeting
-2) Bật camera</t>
-  </si>
-  <si>
-    <t>App hướng dẫn cấp quyền; user vẫn có thể join với audio-only; label/mute/video-off đúng.</t>
+2) Try to enable camera</t>
+  </si>
+  <si>
+    <t>App guides the user to enable permissions; user can still stay in meeting with video off; UI shows correct video-off indicators.</t>
   </si>
   <si>
     <t>JOIN-010</t>
   </si>
   <si>
-    <t>Chọn thiết bị mic/cam/speaker khác trong pre-join và join thành công</t>
-  </si>
-  <si>
-    <t>Máy có &gt;=2 audio devices (hoặc virtual devices); open time đã đến.</t>
+    <t>Select mic/camera/speaker devices in pre-join and join successfully</t>
+  </si>
+  <si>
+    <t>Machine has multiple audio devices or virtual devices; attendee open time has started.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Join
-2) Chọn mic/cam/speaker
-3) Join meeting</t>
-  </si>
-  <si>
-    <t>Thiết bị được áp dụng; âm thanh/video hoạt động; không bị reset khi vào phòng.</t>
+2) Select mic/camera/speaker
+3) Enter the meeting</t>
+  </si>
+  <si>
+    <t>Selected devices are applied; audio/video works; device choice is not reset upon joining.</t>
   </si>
   <si>
     <t>JOIN-011</t>
@@ -269,34 +269,34 @@
     <t>Organizer</t>
   </si>
   <si>
-    <t>Organizer assign Host/Speaker trong Session Editor và user join nhận đúng role</t>
-  </si>
-  <si>
-    <t>Session type Meeting (Collaborative) BETA; organizer đã assign Host + Speaker; open time phù hợp.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Host join
-2) Speaker join
-3) Kiểm tra UI/permissions từng role</t>
-  </si>
-  <si>
-    <t>Host có control host; Speaker có quyền speaker; Attendee không có quyền host. Name labels/role badge đúng.</t>
+    <t>Organizer assigns Host/Speaker; users join and receive correct roles and permissions</t>
+  </si>
+  <si>
+    <t>Session type = Meeting (Collaborative) BETA; organizer assigned host + speaker; joining time window allows entry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Host joins
+2) Speaker joins
+3) Verify UI/permissions per role</t>
+  </si>
+  <si>
+    <t>Host sees host controls; speaker has speaker permissions; attendee does not get host-only controls. Role badge/name labels are correct.</t>
   </si>
   <si>
     <t>JOIN-012</t>
   </si>
   <si>
-    <t>Attendee không thấy/không dùng được các control dành cho Host (lock/admit/remove/spotlight nếu restricted)</t>
-  </si>
-  <si>
-    <t>Attendee joined; host present.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Mở menu controls
-2) Tìm các action host-only</t>
-  </si>
-  <si>
-    <t>Không hiển thị hoặc disabled; không thể gọi API hành động host-only.</t>
+    <t>Attendee cannot access host-only actions (lock/admit/remove/spotlight) if restricted</t>
+  </si>
+  <si>
+    <t>Attendee joined; host is present.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Open meeting controls/menus
+2) Look for host-only actions</t>
+  </si>
+  <si>
+    <t>Host-only actions are hidden or disabled; attendee cannot perform host-only operations via UI/API.</t>
   </si>
   <si>
     <t>JOIN-013</t>
@@ -305,66 +305,66 @@
     <t>Room Lock &amp; Admit</t>
   </si>
   <si>
-    <t>Organizer bật “Lock room” trong Session Editor; attendee join đi vào waiting state</t>
-  </si>
-  <si>
-    <t>Lock room enabled; host assigned; open time đã đến.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Host join
-2) Attendee join</t>
-  </si>
-  <si>
-    <t>Attendee không vào ngay; vào trạng thái chờ (waiting room) hoặc thông báo “Waiting for admission”. Host thấy danh sách chờ.</t>
+    <t>Organizer enables “Lock room” in Session Editor; attendee join goes to a waiting state</t>
+  </si>
+  <si>
+    <t>Lock room is enabled; host assigned; attendee open time has started.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Host joins
+2) Attendee joins</t>
+  </si>
+  <si>
+    <t>Attendee does not enter immediately; sees waiting/admission UI. Host sees a pending admissions list.</t>
   </si>
   <si>
     <t>JOIN-014</t>
   </si>
   <si>
-    <t>Host admit từng attendee khi room locked</t>
-  </si>
-  <si>
-    <t>Room locked; có 2 attendee đang chờ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Host mở danh sách waiting
+    <t>Host admits attendees individually when room is locked</t>
+  </si>
+  <si>
+    <t>Room locked; two attendees are waiting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Host opens waiting list
 2) Admit attendee A
-3) Từ chối/giữ lại attendee B</t>
-  </si>
-  <si>
-    <t>Attendee A vào phòng và xuất hiện trong people roster; attendee B vẫn ở trạng thái chờ; participant count cập nhật đúng.</t>
+3) Keep attendee B waiting (or deny if supported)</t>
+  </si>
+  <si>
+    <t>Attendee A enters and appears in people roster; attendee B remains waiting; participant count updates correctly.</t>
   </si>
   <si>
     <t>JOIN-015</t>
   </si>
   <si>
-    <t>Host lock room trong meeting (nếu có control) và attendee join sau đó bị chặn + vào waiting</t>
-  </si>
-  <si>
-    <t>Host in meeting; room initially unlocked; open time đã đến.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Host bật Lock
-2) Attendee mới join</t>
-  </si>
-  <si>
-    <t>Attendee mới không vào thẳng; host thấy pending admit.</t>
+    <t>If host locks the room in-meeting (if supported), new joiners are routed to waiting/admission flow</t>
+  </si>
+  <si>
+    <t>Host is in the meeting; room initially unlocked; attendee open time has started.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Host enables Lock
+2) New attendee attempts to join</t>
+  </si>
+  <si>
+    <t>New attendee does not enter directly; host sees pending admission.</t>
   </si>
   <si>
     <t>JOIN-016</t>
   </si>
   <si>
-    <t>Attendee bị giữ ở waiting: refresh tab vẫn giữ trạng thái chờ đúng</t>
-  </si>
-  <si>
-    <t>Room locked; attendee đang waiting.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Attendee refresh page
-2) Observe status</t>
-  </si>
-  <si>
-    <t>Vẫn ở trạng thái chờ (không bypass lock); không bị join vào phòng nếu chưa admit.</t>
+    <t>Attendee waiting for admission cannot bypass by refreshing the page</t>
+  </si>
+  <si>
+    <t>Room locked; attendee is currently waiting for admission.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Refresh the page
+2) Observe state</t>
+  </si>
+  <si>
+    <t>Attendee remains in waiting state; does not bypass lock; no unauthorized entry.</t>
   </si>
   <si>
     <t>JOIN-017</t>
@@ -373,35 +373,35 @@
     <t>Sharing Matrix</t>
   </si>
   <si>
-    <t>Sharing matrix: cấu hình quyền screenshare cho Host/Speaker/Attendee ảnh hưởng đúng khi user join</t>
-  </si>
-  <si>
-    <t>Set sharing matrix for Screen Share = Host only (ví dụ).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Host join -&gt; thử share screen
-2) Speaker join -&gt; thử
-3) Attendee join -&gt; thử</t>
-  </si>
-  <si>
-    <t>Chỉ role được phép mới share; role khác bị ẩn/disabled và không share được.</t>
+    <t>Sharing matrix: screen share permission enforced by role after joining</t>
+  </si>
+  <si>
+    <t>Sharing matrix set so Screen Share = Host only (example).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Host joins and tries screen share
+2) Speaker joins and tries
+3) Attendee joins and tries</t>
+  </si>
+  <si>
+    <t>Only permitted roles can start screen share; others see control hidden/disabled and cannot share.</t>
   </si>
   <si>
     <t>JOIN-018</t>
   </si>
   <si>
-    <t>Sharing matrix: cấu hình quyền chat (platform/backstage) hoạt động đúng theo role khi join</t>
+    <t>Sharing matrix: chat permissions (in-session/backstage) enforced by role after joining</t>
   </si>
   <si>
     <t>Chat permissions configured in sharing matrix.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Host/Speaker/Attendee join
-2) Thử gửi chat trong session
-3) Thử backstage chat (nếu có)</t>
-  </si>
-  <si>
-    <t>Luồng chat đúng theo cấu hình; user không được phép không thấy hoặc không gửi được.</t>
+2) Try sending in-session chat
+3) Try backstage chat (if available)</t>
+  </si>
+  <si>
+    <t>Chat visibility and send permissions match configuration; unauthorized roles cannot see or cannot send.</t>
   </si>
   <si>
     <t>JOIN-019</t>
@@ -410,51 +410,51 @@
     <t>Audio/Video</t>
   </si>
   <si>
-    <t>Join với mic ON: trạng thái mute hiển thị đúng cho self và người khác</t>
-  </si>
-  <si>
-    <t>Attendee permitted to unmute; device OK.</t>
+    <t>Join with mic ON: mute state is displayed correctly to self and others</t>
+  </si>
+  <si>
+    <t>Attendee is allowed to unmute; devices are working.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Join
-2) Bật mic
-3) Quan sát roster</t>
-  </si>
-  <si>
-    <t>Icon mute/unmute đúng; “Display if a user is Mute” chính xác trên roster và tile.</t>
+2) Enable mic
+3) Observe roster/tile indicators</t>
+  </si>
+  <si>
+    <t>Mute/unmute indicators are correct on roster and tiles ("Display if a user is Mute" works).</t>
   </si>
   <si>
     <t>JOIN-020</t>
   </si>
   <si>
-    <t>Join với mic OFF: default mute và hiển thị đúng</t>
-  </si>
-  <si>
-    <t>Default join setting (nếu có) = mute; open time đã đến.</t>
+    <t>Join with mic OFF: default mute state is correct</t>
+  </si>
+  <si>
+    <t>Default join behavior (if any) results in muted state; attendee open time has started.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Join
-2) Không bật mic</t>
-  </si>
-  <si>
-    <t>Attendee ở trạng thái mute; icon đúng; không phát audio.</t>
+2) Do not enable mic</t>
+  </si>
+  <si>
+    <t>Attendee remains muted; icon is correct; no audio is transmitted.</t>
   </si>
   <si>
     <t>JOIN-021</t>
   </si>
   <si>
-    <t>Bật/tắt webcam trong meeting sau khi join: tile + name label cập nhật đúng</t>
+    <t>Toggle webcam after joining: tile and name label update correctly</t>
   </si>
   <si>
     <t>Attendee joined; camera permission granted.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Bật camera
-2) Tắt camera
-3) Bật lại</t>
-  </si>
-  <si>
-    <t>Video tile cập nhật tức thì; name labels vẫn hiển thị; không bị freeze.</t>
+    <t xml:space="preserve">1) Turn camera on
+2) Turn camera off
+3) Turn camera on again</t>
+  </si>
+  <si>
+    <t>Video tile updates promptly; name labels remain visible; no freezing or stuck video.</t>
   </si>
   <si>
     <t>JOIN-022</t>
@@ -463,33 +463,33 @@
     <t>Capacity (12 webcams)</t>
   </si>
   <si>
-    <t>Tối đa 12 participants bật webcam cùng lúc: user thứ 13 bị chặn/auto video-off theo rule</t>
-  </si>
-  <si>
-    <t>Có &gt;=13 users join cùng session; policy max webcam=12.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Cho 12 users bật camera
-2) User thứ 13 bật camera</t>
-  </si>
-  <si>
-    <t>Hệ thống enforce giới hạn: user #13 không bật được hoặc tự chuyển sang video-off + message rõ ràng; không ảnh hưởng 12 user còn lại.</t>
+    <t>Max 12 participants can have webcams ON simultaneously; participant #13 is blocked or forced video-off per rule</t>
+  </si>
+  <si>
+    <t>At least 13 users can join the session; max webcam sharing = 12.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Have 12 users turn on camera
+2) User #13 attempts to turn on camera</t>
+  </si>
+  <si>
+    <t>System enforces the limit: user #13 cannot enable camera or is forced to video-off with a clear message; existing 12 are unaffected.</t>
   </si>
   <si>
     <t>JOIN-023</t>
   </si>
   <si>
-    <t>Khi một trong 12 users tắt camera, user khác có thể bật camera thay thế</t>
-  </si>
-  <si>
-    <t>Đang có 12 cameras ON; 1 user tắt cam.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) User A tắt camera
-2) User B (đang video-off) bật camera</t>
-  </si>
-  <si>
-    <t>User B bật được camera; giới hạn vẫn đúng.</t>
+    <t>When one of the 12 users turns camera off, another user can turn camera on</t>
+  </si>
+  <si>
+    <t>There are 12 cameras ON; one user turns camera OFF.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) User A turns camera off
+2) User B (currently video off) turns camera on</t>
+  </si>
+  <si>
+    <t>User B can enable camera; the limit is still enforced correctly.</t>
   </si>
   <si>
     <t>JOIN-024</t>
@@ -498,51 +498,51 @@
     <t>Chat &amp; People Roster</t>
   </si>
   <si>
-    <t>People list hiển thị đúng số lượng participant + participant count đồng bộ</t>
-  </si>
-  <si>
-    <t>Có nhiều users join/leave.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Mở People
-2) So sánh participant count vs roster
-3) Cho 1 user rời
-4) Kiểm tra lại</t>
-  </si>
-  <si>
-    <t>Số lượng đồng bộ, update gần realtime; không ghost user.</t>
+    <t>People list shows correct participants and participant count stays in sync</t>
+  </si>
+  <si>
+    <t>Multiple users join/leave during the test.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Open People
+2) Compare participant count vs roster
+3) Have a user leave
+4) Re-check</t>
+  </si>
+  <si>
+    <t>Counts are consistent and update near real-time; no ghost/duplicate users.</t>
   </si>
   <si>
     <t>JOIN-025</t>
   </si>
   <si>
-    <t>Session chat gửi/nhận tin nhắn sau khi join</t>
-  </si>
-  <si>
-    <t>Chat enabled theo sharing matrix.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Attendee A gửi tin
-2) Attendee B nhận và reply</t>
-  </si>
-  <si>
-    <t>Tin nhắn hiển thị đúng thứ tự; timestamp/author đúng; không leak giữa session khác.</t>
+    <t>In-session chat send/receive works after joining</t>
+  </si>
+  <si>
+    <t>Chat is enabled in sharing matrix.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Attendee A sends a message
+2) Attendee B receives and replies</t>
+  </si>
+  <si>
+    <t>Messages appear in correct order; author/time metadata is correct; no leakage across sessions.</t>
   </si>
   <si>
     <t>JOIN-026</t>
   </si>
   <si>
-    <t>Lower hand trong people roster khi attendee raise hand</t>
-  </si>
-  <si>
-    <t>Raise hand enabled; attendee joined.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Attendee raise hand
-2) Host lower hand</t>
-  </si>
-  <si>
-    <t>Icon hand raise biến mất; attendee thấy trạng thái bị hạ tay.</t>
+    <t>Host can lower raised hands via people roster</t>
+  </si>
+  <si>
+    <t>Hand raise is enabled; attendee joined.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Attendee raises hand
+2) Host lowers hand</t>
+  </si>
+  <si>
+    <t>Hand raise indicator is cleared for all users; attendee sees the updated state.</t>
   </si>
   <si>
     <t>JOIN-027</t>
@@ -551,18 +551,18 @@
     <t>Reactions &amp; Hand Raise</t>
   </si>
   <si>
-    <t>Emoji reactions (clap/others) hoạt động sau khi join</t>
-  </si>
-  <si>
-    <t>Reactions enabled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Attendee gửi clap
-2) Quan sát tile/overlay
-3) Người khác nhìn thấy</t>
-  </si>
-  <si>
-    <t>Reaction hiển thị đúng UI; không spam vượt rate limit (nếu có); không ảnh hưởng audio/video.</t>
+    <t>Emoji reactions (clap and others) work after joining</t>
+  </si>
+  <si>
+    <t>Reactions are enabled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Attendee sends a clap reaction
+2) Observe overlay on tile
+3) Confirm other participants can see it</t>
+  </si>
+  <si>
+    <t>Reaction UI displays correctly; does not break audio/video; rate limiting (if any) behaves correctly.</t>
   </si>
   <si>
     <t>JOIN-028</t>
@@ -571,34 +571,34 @@
     <t>Spotlight &amp; Layout (PIP)</t>
   </si>
   <si>
-    <t>Host spotlight một participant; người mới join thấy spotlight state đúng</t>
-  </si>
-  <si>
-    <t>Meeting đang chạy; host đã spotlight Speaker.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Attendee mới join
-2) Quan sát layout</t>
-  </si>
-  <si>
-    <t>Attendee mới join thấy participant đang spotlight theo state hiện tại; không reset.</t>
+    <t>Host spotlights a participant; users who join later see the correct spotlight state</t>
+  </si>
+  <si>
+    <t>Meeting is live; host has spotlighted a speaker.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) New attendee joins
+2) Observe layout</t>
+  </si>
+  <si>
+    <t>New attendee sees the same spotlight state; spotlight is not reset on join.</t>
   </si>
   <si>
     <t>JOIN-029</t>
   </si>
   <si>
-    <t>Dynamic PIP mode hoạt động khi user join và share screen (nếu được phép)</t>
-  </si>
-  <si>
-    <t>Sharing matrix cho phép; user joined.</t>
+    <t>Dynamic PIP mode behaves correctly when joining and starting screen share (if permitted)</t>
+  </si>
+  <si>
+    <t>Sharing matrix permits user to share screen; user has joined.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Start screen share
-2) Quan sát PIP
-3) Tắt share</t>
-  </si>
-  <si>
-    <t>PIP chuyển đổi mượt; không che controls; stop share trả layout về bình thường.</t>
+2) Observe PIP layout
+3) Stop share</t>
+  </si>
+  <si>
+    <t>PIP transitions smoothly; does not block controls; layout returns correctly after stopping share.</t>
   </si>
   <si>
     <t>JOIN-030</t>
@@ -607,17 +607,17 @@
     <t>Remove User &amp; Moderation</t>
   </si>
   <si>
-    <t>Host remove một attendee khỏi meeting; attendee bị kick và không tự vào lại nếu bị chặn theo rule</t>
-  </si>
-  <si>
-    <t>Attendee joined; host has permission.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Host remove attendee
-2) Attendee cố join lại ngay</t>
-  </si>
-  <si>
-    <t>Attendee bị out; khi join lại: (a) bị chặn nếu policy “removed” hoặc (b) phải re-admit nếu room locked; không tự bypass.</t>
+    <t>Host removes an attendee; attendee is kicked and cannot bypass by immediate rejoin</t>
+  </si>
+  <si>
+    <t>Attendee joined; host has permission to remove.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Host removes attendee
+2) Attendee attempts to rejoin immediately</t>
+  </si>
+  <si>
+    <t>Attendee is removed; rejoin behavior follows policy (blocked/needs admission if locked); no bypass.</t>
   </si>
   <si>
     <t>JOIN-031</t>
@@ -626,53 +626,53 @@
     <t>Recording Controls</t>
   </si>
   <si>
-    <t>Nếu “Allow session to be recorded” OFF: không ai thấy nút start/stop recording khi live</t>
-  </si>
-  <si>
-    <t>Session editor: recording checkbox OFF; session live.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Host join
-2) Speaker join
-3) Attendee join
-4) Tìm recording controls</t>
-  </si>
-  <si>
-    <t>Không có control record; không thể start record bằng UI.</t>
+    <t>When “Allow session to be recorded” is OFF: no start/stop recording controls are shown while live</t>
+  </si>
+  <si>
+    <t>Session editor: recording checkbox OFF; session is live.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Host joins
+2) Speaker joins
+3) Attendee joins
+4) Look for recording controls</t>
+  </si>
+  <si>
+    <t>No recording controls are visible; recording cannot be started from the UI.</t>
   </si>
   <si>
     <t>JOIN-032</t>
   </si>
   <si>
-    <t>Nếu “Allow session to be recorded” ON: organizer/host (theo spec) thấy nút start recording khi session live</t>
-  </si>
-  <si>
-    <t>Recording checkbox ON; session live; xác định role nào được record theo thiết kế.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Host join
-2) Tìm nút Start Recording
-3) Start
-4) Stop</t>
-  </si>
-  <si>
-    <t>Start/Stop hoạt động; trạng thái recording hiển thị; không ảnh hưởng join của participants.</t>
+    <t>When “Allow session to be recorded” is ON: permitted roles can start/stop recording while live</t>
+  </si>
+  <si>
+    <t>Recording checkbox ON; session is live; confirm which roles are permitted to control recording.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Join as a permitted role
+2) Click Start Recording
+3) Verify recording state
+4) Click Stop Recording</t>
+  </si>
+  <si>
+    <t>Start/Stop works; recording state indicator is correct; joining participants are not disrupted.</t>
   </si>
   <si>
     <t>JOIN-033</t>
   </si>
   <si>
-    <t>Attendee không có quyền start/stop recording</t>
-  </si>
-  <si>
-    <t>Recording enabled; attendee joined.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Mở controls
-2) Tìm record</t>
-  </si>
-  <si>
-    <t>Không hiển thị hoặc disabled; không trigger recording.</t>
+    <t>Attendee cannot start/stop recording</t>
+  </si>
+  <si>
+    <t>Recording is enabled; attendee joined.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Open meeting controls
+2) Look for recording actions</t>
+  </si>
+  <si>
+    <t>Recording controls are hidden/disabled for attendee; attendee cannot start recording via UI/API.</t>
   </si>
   <si>
     <t>JOIN-034</t>
@@ -681,18 +681,18 @@
     <t>Localization (10 languages)</t>
   </si>
   <si>
-    <t>Join meeting với UI language khác (trong 10 ngôn ngữ) không vỡ layout và strings đúng</t>
-  </si>
-  <si>
-    <t>Set language = non-default (ví dụ: FR/DE/JA); open time đã đến.</t>
+    <t>Join meeting in a non-default UI language: strings are correct and layout is not broken</t>
+  </si>
+  <si>
+    <t>Set UI language to a supported non-default language (e.g., FR/DE/JA); attendee open time has started.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Join
-2) Mở People/Chat/Reactions
-3) Observe labels</t>
-  </si>
-  <si>
-    <t>Text dịch đúng; không tràn UI; join flow không lỗi.</t>
+2) Open People/Chat/Reactions
+3) Review labels and layout</t>
+  </si>
+  <si>
+    <t>Translations are correct; no text overflow or broken layouts; join flow works without errors.</t>
   </si>
   <si>
     <t>P2</t>
@@ -704,36 +704,36 @@
     <t>Resilience (reconnect)</t>
   </si>
   <si>
-    <t>Mất mạng ngắn (10-30s) rồi reconnect: user giữ được state hợp lý (mute/cam/hand raise) và không nhân đôi trong roster</t>
-  </si>
-  <si>
-    <t>Attendee joined; network throttling available.</t>
+    <t>Short network drop (10–30s) then reconnect: no duplicate roster entries and state remains reasonable</t>
+  </si>
+  <si>
+    <t>Attendee joined; network throttling can be simulated.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Join
-2) Bật cam
-3) Ngắt mạng 20s
-4) Bật lại
-5) Quan sát roster/chat</t>
-  </si>
-  <si>
-    <t>Tự reconnect; không duplicate user; trạng thái audio/video phục hồi theo rule; chat vẫn dùng được sau reconnect.</t>
+2) Turn camera on
+3) Disable network for 20s
+4) Re-enable network
+5) Observe roster and chat</t>
+  </si>
+  <si>
+    <t>Client reconnects automatically; no duplicate/ghost users; audio/video state follows defined rules; chat still works after reconnect.</t>
   </si>
   <si>
     <t>JOIN-036</t>
   </si>
   <si>
-    <t>Refresh tab khi đang trong meeting: rejoin thành công và state hiển thị đúng</t>
-  </si>
-  <si>
-    <t>Attendee joined; room unlocked hoặc locked với auto-rejoin rule.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Refresh
-2) Observe</t>
-  </si>
-  <si>
-    <t>User quay lại meeting; nếu room locked thì xử lý đúng (re-admit nếu cần); không crash.</t>
+    <t>Refresh browser tab while in meeting: rejoin works and lock-room rules are respected</t>
+  </si>
+  <si>
+    <t>Attendee joined; room is unlocked OR locked with an admission policy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Refresh the tab
+2) Observe join behavior</t>
+  </si>
+  <si>
+    <t>User returns to meeting; if room is locked the correct admission flow is applied; no crash.</t>
   </si>
   <si>
     <t>JOIN-037</t>
@@ -742,118 +742,118 @@
     <t>Reporting (attendance/dwell)</t>
   </si>
   <si>
-    <t>Attendance report có dwell time: join/leave nhiều lần vẫn tính đúng dwell time tổng</t>
-  </si>
-  <si>
-    <t>Reporting enabled; organizer access to reports.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Attendee join 5 phút
-2) Leave 2 phút
-3) Join lại 3 phút
-4) Export/view report</t>
-  </si>
-  <si>
-    <t>Dwell time tổng = 8 phút (± rounding); không double count sessions.</t>
+    <t>Attendance report includes dwell time: multiple joins/leaves aggregate correctly</t>
+  </si>
+  <si>
+    <t>Reporting is enabled; organizer can access attendance report.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Attendee joins for 5 minutes
+2) Leaves for 2 minutes
+3) Joins again for 3 minutes
+4) View/export report</t>
+  </si>
+  <si>
+    <t>Total dwell time is 8 minutes (± rounding); not double-counted.</t>
   </si>
   <si>
     <t>JOIN-038</t>
   </si>
   <si>
-    <t>Join đúng giờ nhưng session đã kết thúc: hiển thị trạng thái ended + CTA xem recording (nếu có)</t>
-  </si>
-  <si>
-    <t>Session ended; recordings maybe available.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Attendee mở Agenda
-2) Nhấn Join</t>
-  </si>
-  <si>
-    <t>Không vào meeting live; hiển thị ended; nếu recording available thì CTA xem recording đúng.</t>
+    <t>Attempt to join after session ended: shows ended state and (optionally) recording CTA</t>
+  </si>
+  <si>
+    <t>Session is ended; recording may or may not be available.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Open Agenda
+2) Click Join</t>
+  </si>
+  <si>
+    <t>User cannot enter live meeting; ended state is shown; if recording is available, CTA to view recording is correct.</t>
   </si>
   <si>
     <t>JOIN-039</t>
   </si>
   <si>
-    <t>Join link mở ở 2 tabs: tab thứ 2 xử lý đúng (deny / takeover) theo policy</t>
-  </si>
-  <si>
-    <t>Attendee has meeting open in Tab A.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Mở Tab B cùng join link
+    <t>Open the same join link in two tabs: policy prevents duplicate participants</t>
+  </si>
+  <si>
+    <t>Attendee already joined in Tab A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Open Tab B with the same join link
 2) Observe behavior</t>
   </si>
   <si>
-    <t>Không tạo 2 participants trùng; xử lý rõ ràng (ví dụ: kick session cũ hoặc chặn session mới).</t>
+    <t>System prevents duplicate participant sessions; behavior is clear (deny new tab or transfer session).</t>
   </si>
   <si>
     <t>JOIN-040</t>
   </si>
   <si>
-    <t>Name labels hiển thị đúng với ký tự Unicode (tiếng Việt/JP/emoji) khi user join</t>
-  </si>
-  <si>
-    <t>User display name chứa Unicode (ví dụ: “Nguyễn Ánh – 山田”).</t>
+    <t>Name labels render correctly for Unicode (Vietnamese diacritics/CJK) when joining</t>
+  </si>
+  <si>
+    <t>User display name contains Unicode (e.g., “Nguyễn Ánh – 山田”).</t>
   </si>
   <si>
     <t xml:space="preserve">1) Join
-2) Quan sát name label trên tile + people list</t>
-  </si>
-  <si>
-    <t>Không lỗi encoding; không cắt sai; hiển thị nhất quán.</t>
+2) Observe name label on tiles and in people roster</t>
+  </si>
+  <si>
+    <t>No encoding issues; consistent rendering; no incorrect truncation.</t>
   </si>
   <si>
     <t>JOIN-041</t>
   </si>
   <si>
-    <t>Set Avatar trước khi join: nếu video-off thì avatar hiển thị thay thế đúng</t>
-  </si>
-  <si>
-    <t>User set avatar; join với camera off.</t>
+    <t>Avatar is shown when user joins with camera off (after setting an avatar)</t>
+  </si>
+  <si>
+    <t>User has set an avatar; user joins with camera off.</t>
   </si>
   <si>
     <t xml:space="preserve">1) Join
-2) Camera off
+2) Ensure camera is off
 3) Observe tile</t>
   </si>
   <si>
-    <t>Avatar hiển thị thay video; name label vẫn có; không dùng avatar của user khác.</t>
+    <t>Avatar is shown as the placeholder; name label remains correct; no avatar mix-ups.</t>
   </si>
   <si>
     <t>JOIN-042</t>
   </si>
   <si>
-    <t>Backstage chat (nếu có) chỉ thấy giữa participants được phép (Host/Speaker) khi join</t>
-  </si>
-  <si>
-    <t>Backstage chat enabled; attendee joined too.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Speaker gửi backstage chat
-2) Host nhận
-3) Attendee kiểm tra chat</t>
-  </si>
-  <si>
-    <t>Attendee không thấy backstage messages; host/speaker thấy đúng.</t>
+    <t>Backstage chat (if available) is only visible to permitted roles (Host/Speaker) when joining</t>
+  </si>
+  <si>
+    <t>Backstage chat enabled; at least one attendee is also in the meeting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Speaker sends backstage message
+2) Host verifies receipt
+3) Attendee checks chat</t>
+  </si>
+  <si>
+    <t>Attendee cannot see backstage messages; host/speaker can.</t>
   </si>
   <si>
     <t>JOIN-043</t>
   </si>
   <si>
-    <t>Video share (YouTube): user join sau khi video đang share vẫn thấy playback/state đúng</t>
-  </si>
-  <si>
-    <t>Host đang share YouTube; sharing allowed; attendee join sau.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Host share YouTube
-2) Attendee join
-3) Observe</t>
-  </si>
-  <si>
-    <t>Attendee mới join thấy video share; sync state (play/pause) theo rule; audio mix không lỗi.</t>
+    <t>YouTube video share: users who join after sharing starts see correct playback/state</t>
+  </si>
+  <si>
+    <t>Host is sharing a YouTube video; sharing is permitted; attendee joins afterward.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Host starts YouTube share
+2) Attendee joins
+3) Observe video and audio</t>
+  </si>
+  <si>
+    <t>Late joiner sees the shared video; state (play/pause) aligns with the meeting per policy; no audio issues.</t>
   </si>
   <si>
     <t>Setting / Capability</t>
@@ -868,16 +868,16 @@
     <t>No</t>
   </si>
   <si>
-    <t>Available when “Enable Virtual session” toggled ON.</t>
+    <t>Available when “Enable Virtual session” is toggled ON.</t>
   </si>
   <si>
     <t>Assign hosts/speakers in Session Editor</t>
   </si>
   <si>
-    <t>Verify role mapping reflected when users join.</t>
-  </si>
-  <si>
-    <t>Host start time (can start 4h early)</t>
+    <t>Verify role mapping is reflected when users join.</t>
+  </si>
+  <si>
+    <t>Host early start (can start 4h early)</t>
   </si>
   <si>
     <t>Config</t>
@@ -910,10 +910,10 @@
     <t>If locked, hosts admit participants manually.</t>
   </si>
   <si>
-    <t>Admit participants when room locked</t>
-  </si>
-  <si>
-    <t>Verify waiting room UX on join.</t>
+    <t>Admit participants when room is locked</t>
+  </si>
+  <si>
+    <t>Validate waiting room UX on join.</t>
   </si>
   <si>
     <t>Sharing access (screen share/chat/video share) via Sharing Matrix</t>
@@ -922,13 +922,13 @@
     <t>Per config</t>
   </si>
   <si>
-    <t>Core join-related validation: controls visible/enforced by role.</t>
+    <t>Join-related validation: controls visibility and enforcement by role.</t>
   </si>
   <si>
     <t>Allow session to be recorded (checkbox in Session Editor)</t>
   </si>
   <si>
-    <t>When enabled: start/stop recording option appears when live (role TBD by product).</t>
+    <t>When enabled: start/stop recording option appears when live (permitted role TBD by product).</t>
   </si>
   <si>
     <t>Data Type</t>
@@ -943,7 +943,7 @@
     <t>Chrome / Edge / Firefox / Safari</t>
   </si>
   <si>
-    <t>Test join flow + permissions prompts; Safari for AV quirks.</t>
+    <t>Validate join flow + permissions prompts; include Safari for AV edge cases.</t>
   </si>
   <si>
     <t>Devices</t>
@@ -952,7 +952,7 @@
     <t>Desktop + Mobile</t>
   </si>
   <si>
-    <t>If mobile supported, validate join/AV UI responsive.</t>
+    <t>If mobile is supported, validate join and responsive UI.</t>
   </si>
   <si>
     <t>Network</t>
@@ -961,7 +961,7 @@
     <t>Good / Poor / Drop 20s</t>
   </si>
   <si>
-    <t>Reconnect + roster dedupe + chat continuity.</t>
+    <t>Reconnect behavior + roster dedupe + chat continuity.</t>
   </si>
   <si>
     <t>Accounts</t>
@@ -970,7 +970,7 @@
     <t>Host_1, Speaker_1, Attendee_1..14</t>
   </si>
   <si>
-    <t>Need 13+ to verify 12 webcam limit.</t>
+    <t>Need 13+ users to validate 12 webcam limit.</t>
   </si>
   <si>
     <t>Names</t>
@@ -979,7 +979,7 @@
     <t>Unicode names</t>
   </si>
   <si>
-    <t>Vietnamese diacritics + CJK; validate labels.</t>
+    <t>Vietnamese diacritics + CJK; validate labels in tiles and roster.</t>
   </si>
   <si>
     <t>Languages</t>
@@ -988,7 +988,7 @@
     <t>10 supported languages</t>
   </si>
   <si>
-    <t>Pick 2-3 representative (EN, FR/DE, JA/KR) for UI overflow.</t>
+    <t>Pick 2–3 representative languages to verify layout and translations.</t>
   </si>
   <si>
     <t>Field</t>
@@ -1003,25 +1003,25 @@
     <t>Not Run, Pass, Fail, Blocked, N/A</t>
   </si>
   <si>
-    <t>Checklist execution status for each test case.</t>
+    <t>Execution status per test case.</t>
   </si>
   <si>
     <t>P0, P1, P2, P3</t>
   </si>
   <si>
-    <t>P0=must-pass release blocker; P1=high; P2=medium; P3=low.</t>
+    <t>P0 = release blocker; P1 = high; P2 = medium; P3 = low.</t>
   </si>
   <si>
     <t>Host, Speaker, Attendee, Organizer, Co-host, Unknown/Guest</t>
   </si>
   <si>
-    <t>Primary user role for the test scenario.</t>
+    <t>Primary user role for the scenario.</t>
   </si>
   <si>
     <t>Access &amp; Timing, Agenda Lobby Entry, Pre-join &amp; Device Checks, Role &amp; Permissions, Room Lock &amp; Admit, Sharing Matrix, Audio/Video, Capacity (12 webcams), Chat &amp; People Roster, Reactions &amp; Hand Raise, Spotlight &amp; Layout (PIP), Remove User &amp; Moderation, Recording Controls, Localization (10 languages), Resilience (reconnect), Reporting (attendance/dwell)</t>
   </si>
   <si>
-    <t>Functional area grouping (focused on join).</t>
+    <t>Functional grouping (join-focused).</t>
   </si>
 </sst>
 </file>
@@ -1561,7 +1561,7 @@
         <v>29</v>
       </c>
       <c r="H3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I3" t="s">
         <v>22</v>
@@ -1584,28 +1584,28 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>36</v>
-      </c>
       <c r="H4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I4" t="s">
         <v>22</v>
@@ -1628,28 +1628,28 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>41</v>
-      </c>
       <c r="H5" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I5" t="s">
         <v>22</v>
@@ -1672,28 +1672,28 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" t="s">
         <v>46</v>
-      </c>
-      <c r="H6" t="s">
-        <v>21</v>
       </c>
       <c r="I6" t="s">
         <v>22</v>
@@ -1722,7 +1722,7 @@
         <v>49</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>50</v>
@@ -1737,7 +1737,7 @@
         <v>53</v>
       </c>
       <c r="H7" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I7" t="s">
         <v>22</v>
@@ -1781,7 +1781,7 @@
         <v>59</v>
       </c>
       <c r="H8" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I8" t="s">
         <v>60</v>
@@ -1810,7 +1810,7 @@
         <v>62</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>63</v>
@@ -1825,7 +1825,7 @@
         <v>66</v>
       </c>
       <c r="H9" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I9" t="s">
         <v>22</v>
@@ -1854,7 +1854,7 @@
         <v>62</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>68</v>
@@ -1869,7 +1869,7 @@
         <v>71</v>
       </c>
       <c r="H10" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I10" t="s">
         <v>22</v>
@@ -1898,7 +1898,7 @@
         <v>62</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>73</v>
@@ -1913,7 +1913,7 @@
         <v>76</v>
       </c>
       <c r="H11" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I11" t="s">
         <v>22</v>
@@ -1957,7 +1957,7 @@
         <v>83</v>
       </c>
       <c r="H12" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I12" t="s">
         <v>22</v>
@@ -1986,7 +1986,7 @@
         <v>78</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>85</v>
@@ -2001,7 +2001,7 @@
         <v>88</v>
       </c>
       <c r="H13" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I13" t="s">
         <v>60</v>
@@ -2045,7 +2045,7 @@
         <v>94</v>
       </c>
       <c r="H14" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I14" t="s">
         <v>22</v>
@@ -2089,7 +2089,7 @@
         <v>99</v>
       </c>
       <c r="H15" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I15" t="s">
         <v>22</v>
@@ -2133,7 +2133,7 @@
         <v>104</v>
       </c>
       <c r="H16" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I16" t="s">
         <v>22</v>
@@ -2162,7 +2162,7 @@
         <v>90</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>106</v>
@@ -2177,7 +2177,7 @@
         <v>109</v>
       </c>
       <c r="H17" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I17" t="s">
         <v>60</v>
@@ -2221,7 +2221,7 @@
         <v>115</v>
       </c>
       <c r="H18" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I18" t="s">
         <v>22</v>
@@ -2265,7 +2265,7 @@
         <v>120</v>
       </c>
       <c r="H19" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I19" t="s">
         <v>22</v>
@@ -2294,7 +2294,7 @@
         <v>122</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>123</v>
@@ -2309,7 +2309,7 @@
         <v>126</v>
       </c>
       <c r="H20" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I20" t="s">
         <v>22</v>
@@ -2338,7 +2338,7 @@
         <v>122</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>128</v>
@@ -2353,7 +2353,7 @@
         <v>131</v>
       </c>
       <c r="H21" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I21" t="s">
         <v>22</v>
@@ -2382,7 +2382,7 @@
         <v>122</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>133</v>
@@ -2397,7 +2397,7 @@
         <v>136</v>
       </c>
       <c r="H22" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I22" t="s">
         <v>22</v>
@@ -2441,7 +2441,7 @@
         <v>142</v>
       </c>
       <c r="H23" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I23" t="s">
         <v>22</v>
@@ -2470,7 +2470,7 @@
         <v>138</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>144</v>
@@ -2485,7 +2485,7 @@
         <v>147</v>
       </c>
       <c r="H24" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I24" t="s">
         <v>22</v>
@@ -2514,7 +2514,7 @@
         <v>149</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>150</v>
@@ -2529,7 +2529,7 @@
         <v>153</v>
       </c>
       <c r="H25" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I25" t="s">
         <v>22</v>
@@ -2558,7 +2558,7 @@
         <v>149</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>155</v>
@@ -2573,7 +2573,7 @@
         <v>158</v>
       </c>
       <c r="H26" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I26" t="s">
         <v>22</v>
@@ -2617,7 +2617,7 @@
         <v>163</v>
       </c>
       <c r="H27" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I27" t="s">
         <v>22</v>
@@ -2646,7 +2646,7 @@
         <v>165</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>166</v>
@@ -2661,7 +2661,7 @@
         <v>169</v>
       </c>
       <c r="H28" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I28" t="s">
         <v>22</v>
@@ -2705,7 +2705,7 @@
         <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I29" t="s">
         <v>22</v>
@@ -2734,7 +2734,7 @@
         <v>171</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>177</v>
@@ -2749,7 +2749,7 @@
         <v>180</v>
       </c>
       <c r="H30" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I30" t="s">
         <v>22</v>
@@ -2793,7 +2793,7 @@
         <v>186</v>
       </c>
       <c r="H31" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I31" t="s">
         <v>22</v>
@@ -2837,7 +2837,7 @@
         <v>192</v>
       </c>
       <c r="H32" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I32" t="s">
         <v>22</v>
@@ -2881,7 +2881,7 @@
         <v>197</v>
       </c>
       <c r="H33" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I33" t="s">
         <v>22</v>
@@ -2910,7 +2910,7 @@
         <v>188</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>199</v>
@@ -2925,7 +2925,7 @@
         <v>202</v>
       </c>
       <c r="H34" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I34" t="s">
         <v>60</v>
@@ -2954,7 +2954,7 @@
         <v>204</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>205</v>
@@ -2998,7 +2998,7 @@
         <v>211</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>212</v>
@@ -3013,7 +3013,7 @@
         <v>215</v>
       </c>
       <c r="H36" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I36" t="s">
         <v>22</v>
@@ -3042,7 +3042,7 @@
         <v>211</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>217</v>
@@ -3057,7 +3057,7 @@
         <v>220</v>
       </c>
       <c r="H37" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I37" t="s">
         <v>22</v>
@@ -3101,7 +3101,7 @@
         <v>226</v>
       </c>
       <c r="H38" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I38" t="s">
         <v>22</v>
@@ -3130,7 +3130,7 @@
         <v>15</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>228</v>
@@ -3145,7 +3145,7 @@
         <v>231</v>
       </c>
       <c r="H39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I39" t="s">
         <v>22</v>
@@ -3174,7 +3174,7 @@
         <v>49</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>233</v>
@@ -3189,7 +3189,7 @@
         <v>236</v>
       </c>
       <c r="H40" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I40" t="s">
         <v>22</v>
@@ -3218,7 +3218,7 @@
         <v>149</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>238</v>
@@ -3262,7 +3262,7 @@
         <v>122</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>243</v>
@@ -3306,7 +3306,7 @@
         <v>149</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>248</v>
@@ -3321,7 +3321,7 @@
         <v>251</v>
       </c>
       <c r="H43" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I43" t="s">
         <v>60</v>
@@ -3440,10 +3440,10 @@
         <v>16</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>13</v>

</xml_diff>